<commit_message>
Align field sample numbering with manuscript Table 2
</commit_message>
<xml_diff>
--- a/CaseSamplingData.xlsx
+++ b/CaseSamplingData.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="1" r:id="Ra6fd0420cc2f4836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="2" r:id="R8b28cbb4f6984ddf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="1" r:id="R04aa051e04a24479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dictionary" sheetId="2" r:id="R3c3fc006a6d64a1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -822,37 +822,37 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B13" s="9" t="n">
-        <x:v>9</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="11" t="str">
-        <x:v>train</x:v>
+        <x:v>validation</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
-        <x:v>3-1 Clay</x:v>
+        <x:v>2-2 Clay</x:v>
       </x:c>
       <x:c r="E13" s="13" t="n">
-        <x:v>3056757.95</x:v>
+        <x:v>3056835.92</x:v>
       </x:c>
       <x:c r="F13" s="13" t="n">
-        <x:v>376939.03</x:v>
+        <x:v>376867.39</x:v>
       </x:c>
       <x:c r="G13" s="13" t="n">
-        <x:v>1937.45</x:v>
+        <x:v>1928.02</x:v>
       </x:c>
       <x:c r="H13" s="13" t="n">
-        <x:v>25.03</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="I13" s="13" t="n">
-        <x:v>75.1</x:v>
+        <x:v>3.46</x:v>
       </x:c>
       <x:c r="J13" s="13" t="n">
-        <x:v>20.79</x:v>
+        <x:v>11.36</x:v>
       </x:c>
       <x:c r="K13" s="14" t="n">
-        <x:v>58.3</x:v>
+        <x:v>47.2</x:v>
       </x:c>
       <x:c r="L13" s="15" t="n">
-        <x:v>1.708</x:v>
+        <x:v>1.171</x:v>
       </x:c>
       <x:c r="M13"/>
     </x:row>
@@ -861,37 +861,37 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B14" s="9" t="n">
-        <x:v>10</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>train</x:v>
+        <x:v>validation</x:v>
       </x:c>
       <x:c r="D14" s="11" t="str">
-        <x:v>3-1 Clay</x:v>
+        <x:v>2-3 Clay with rock fragments</x:v>
       </x:c>
       <x:c r="E14" s="13" t="n">
-        <x:v>3056856.29</x:v>
+        <x:v>3056827.82</x:v>
       </x:c>
       <x:c r="F14" s="13" t="n">
-        <x:v>377087.93</x:v>
+        <x:v>376981</x:v>
       </x:c>
       <x:c r="G14" s="13" t="n">
-        <x:v>1929.34</x:v>
+        <x:v>1924.2</x:v>
       </x:c>
       <x:c r="H14" s="13" t="n">
-        <x:v>123.37</x:v>
+        <x:v>94.9</x:v>
       </x:c>
       <x:c r="I14" s="13" t="n">
-        <x:v>224</x:v>
+        <x:v>117.07</x:v>
       </x:c>
       <x:c r="J14" s="13" t="n">
-        <x:v>12.68</x:v>
+        <x:v>7.54</x:v>
       </x:c>
       <x:c r="K14" s="14" t="n">
-        <x:v>52.1</x:v>
+        <x:v>35.1</x:v>
       </x:c>
       <x:c r="L14" s="15" t="n">
-        <x:v>1.639</x:v>
+        <x:v>0.901</x:v>
       </x:c>
       <x:c r="M14"/>
     </x:row>
@@ -900,37 +900,37 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B15" s="9" t="n">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C15" s="11" t="str">
-        <x:v>train</x:v>
+        <x:v>validation</x:v>
       </x:c>
       <x:c r="D15" s="11" t="str">
-        <x:v>3-1 Clay</x:v>
+        <x:v>2-3 Clay with rock fragments</x:v>
       </x:c>
       <x:c r="E15" s="13" t="n">
-        <x:v>3056839.09</x:v>
+        <x:v>3056816.06</x:v>
       </x:c>
       <x:c r="F15" s="13" t="n">
-        <x:v>377131.62</x:v>
+        <x:v>377023.05</x:v>
       </x:c>
       <x:c r="G15" s="13" t="n">
-        <x:v>1926.75</x:v>
+        <x:v>1918.2</x:v>
       </x:c>
       <x:c r="H15" s="13" t="n">
-        <x:v>106.17</x:v>
+        <x:v>83.14</x:v>
       </x:c>
       <x:c r="I15" s="13" t="n">
-        <x:v>267.69</x:v>
+        <x:v>159.12</x:v>
       </x:c>
       <x:c r="J15" s="13" t="n">
-        <x:v>10.09</x:v>
+        <x:v>1.54</x:v>
       </x:c>
       <x:c r="K15" s="14" t="n">
-        <x:v>50.4</x:v>
+        <x:v>40.3</x:v>
       </x:c>
       <x:c r="L15" s="15" t="n">
-        <x:v>1.693</x:v>
+        <x:v>1.19</x:v>
       </x:c>
       <x:c r="M15"/>
     </x:row>
@@ -939,37 +939,37 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B16" s="9" t="n">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="11" t="str">
         <x:v>train</x:v>
       </x:c>
       <x:c r="D16" s="11" t="str">
-        <x:v>3-2 Clay</x:v>
+        <x:v>3-1 Clay</x:v>
       </x:c>
       <x:c r="E16" s="13" t="n">
-        <x:v>3056732.92</x:v>
+        <x:v>3056757.95</x:v>
       </x:c>
       <x:c r="F16" s="13" t="n">
-        <x:v>376990.55</x:v>
+        <x:v>376939.03</x:v>
       </x:c>
       <x:c r="G16" s="13" t="n">
-        <x:v>1927.8</x:v>
+        <x:v>1937.45</x:v>
       </x:c>
       <x:c r="H16" s="13" t="n">
-        <x:v>0</x:v>
+        <x:v>25.03</x:v>
       </x:c>
       <x:c r="I16" s="13" t="n">
-        <x:v>126.62</x:v>
+        <x:v>75.1</x:v>
       </x:c>
       <x:c r="J16" s="13" t="n">
-        <x:v>11.14</x:v>
+        <x:v>20.79</x:v>
       </x:c>
       <x:c r="K16" s="14" t="n">
-        <x:v>55</x:v>
+        <x:v>58.3</x:v>
       </x:c>
       <x:c r="L16" s="15" t="n">
-        <x:v>1.528</x:v>
+        <x:v>1.708</x:v>
       </x:c>
       <x:c r="M16"/>
     </x:row>
@@ -978,37 +978,37 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B17" s="9" t="n">
-        <x:v>6</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C17" s="11" t="str">
-        <x:v>validation</x:v>
+        <x:v>train</x:v>
       </x:c>
       <x:c r="D17" s="11" t="str">
-        <x:v>2-2 Clay</x:v>
+        <x:v>3-1 Clay</x:v>
       </x:c>
       <x:c r="E17" s="13" t="n">
-        <x:v>3056835.92</x:v>
+        <x:v>3056856.29</x:v>
       </x:c>
       <x:c r="F17" s="13" t="n">
-        <x:v>376867.39</x:v>
+        <x:v>377087.93</x:v>
       </x:c>
       <x:c r="G17" s="13" t="n">
-        <x:v>1928.02</x:v>
+        <x:v>1929.34</x:v>
       </x:c>
       <x:c r="H17" s="13" t="n">
-        <x:v>103</x:v>
+        <x:v>123.37</x:v>
       </x:c>
       <x:c r="I17" s="13" t="n">
-        <x:v>3.46</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="J17" s="13" t="n">
-        <x:v>11.36</x:v>
+        <x:v>12.68</x:v>
       </x:c>
       <x:c r="K17" s="14" t="n">
-        <x:v>47.2</x:v>
+        <x:v>52.1</x:v>
       </x:c>
       <x:c r="L17" s="15" t="n">
-        <x:v>1.171</x:v>
+        <x:v>1.639</x:v>
       </x:c>
       <x:c r="M17"/>
     </x:row>
@@ -1017,37 +1017,37 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B18" s="9" t="n">
-        <x:v>2</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>validation</x:v>
+        <x:v>train</x:v>
       </x:c>
       <x:c r="D18" s="11" t="str">
-        <x:v>2-3 Clay with rock fragments</x:v>
+        <x:v>3-1 Clay</x:v>
       </x:c>
       <x:c r="E18" s="13" t="n">
-        <x:v>3056827.82</x:v>
+        <x:v>3056839.09</x:v>
       </x:c>
       <x:c r="F18" s="13" t="n">
-        <x:v>376981</x:v>
+        <x:v>377131.62</x:v>
       </x:c>
       <x:c r="G18" s="13" t="n">
-        <x:v>1924.2</x:v>
+        <x:v>1926.75</x:v>
       </x:c>
       <x:c r="H18" s="13" t="n">
-        <x:v>94.9</x:v>
+        <x:v>106.17</x:v>
       </x:c>
       <x:c r="I18" s="13" t="n">
-        <x:v>117.07</x:v>
+        <x:v>267.69</x:v>
       </x:c>
       <x:c r="J18" s="13" t="n">
-        <x:v>7.54</x:v>
+        <x:v>10.09</x:v>
       </x:c>
       <x:c r="K18" s="14" t="n">
-        <x:v>35.1</x:v>
+        <x:v>50.4</x:v>
       </x:c>
       <x:c r="L18" s="15" t="n">
-        <x:v>0.901</x:v>
+        <x:v>1.693</x:v>
       </x:c>
       <x:c r="M18"/>
     </x:row>
@@ -1056,37 +1056,37 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B19" s="9" t="n">
-        <x:v>7</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C19" s="11" t="str">
-        <x:v>validation</x:v>
+        <x:v>train</x:v>
       </x:c>
       <x:c r="D19" s="11" t="str">
-        <x:v>2-3 Clay with rock fragments</x:v>
+        <x:v>3-2 Clay</x:v>
       </x:c>
       <x:c r="E19" s="13" t="n">
-        <x:v>3056816.06</x:v>
+        <x:v>3056732.92</x:v>
       </x:c>
       <x:c r="F19" s="13" t="n">
-        <x:v>377023.05</x:v>
+        <x:v>376990.55</x:v>
       </x:c>
       <x:c r="G19" s="13" t="n">
-        <x:v>1918.2</x:v>
+        <x:v>1927.8</x:v>
       </x:c>
       <x:c r="H19" s="13" t="n">
-        <x:v>83.14</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I19" s="13" t="n">
-        <x:v>159.12</x:v>
+        <x:v>126.62</x:v>
       </x:c>
       <x:c r="J19" s="13" t="n">
-        <x:v>1.54</x:v>
+        <x:v>11.14</x:v>
       </x:c>
       <x:c r="K19" s="14" t="n">
-        <x:v>40.3</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="L19" s="15" t="n">
-        <x:v>1.19</x:v>
+        <x:v>1.528</x:v>
       </x:c>
       <x:c r="M19"/>
     </x:row>
@@ -1116,7 +1116,7 @@
         <x:v>sample_no</x:v>
       </x:c>
       <x:c r="B2" s="17" t="str">
-        <x:v>Sample number from 1 to 18, used consistently in all field data and validation partitions</x:v>
+        <x:v>Sample number 1–18 following manuscript Table 2, used in all case data and validation files</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="50" customHeight="1">

</xml_diff>

<commit_message>
Normalize workbook theme names
</commit_message>
<xml_diff>
--- a/CaseSamplingData.xlsx
+++ b/CaseSamplingData.xlsx
@@ -140,9 +140,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -192,7 +192,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>